<commit_message>
errore BES polveri sottili
</commit_message>
<xml_diff>
--- a/data_in/bes_2003_2023/Metadati_IT_ed.2025.xlsx
+++ b/data_in/bes_2003_2023/Metadati_IT_ed.2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisamimmi/Github/bilancio_missione/data_in/bes_2003_2023/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9F0590-C6BF-424D-A384-4CFCE9204DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E8B1104-C83E-6C45-A39D-552FAAEF5105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="920" windowWidth="29920" windowHeight="18560" xr2:uid="{F3D8B165-4EAB-4F6E-8ECB-A8ACBEEC6F1B}"/>
+    <workbookView xWindow="33420" yWindow="-3820" windowWidth="32620" windowHeight="19840" xr2:uid="{F3D8B165-4EAB-4F6E-8ECB-A8ACBEEC6F1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Bes dei territori metadati_it" sheetId="2" r:id="rId1"/>
@@ -1532,17 +1532,17 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1907,13 +1907,13 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="38"/>
+      <c r="I1" s="36"/>
     </row>
     <row r="2" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="35" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="5" t="s">
@@ -1942,7 +1942,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="36"/>
+      <c r="A3" s="35"/>
       <c r="B3" s="11" t="s">
         <v>9</v>
       </c>
@@ -1969,7 +1969,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36"/>
+      <c r="A4" s="35"/>
       <c r="B4" s="11" t="s">
         <v>9</v>
       </c>
@@ -1996,7 +1996,7 @@
       </c>
     </row>
     <row r="5" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="36"/>
+      <c r="A5" s="35"/>
       <c r="B5" s="11" t="s">
         <v>9</v>
       </c>
@@ -2023,7 +2023,7 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="36"/>
+      <c r="A6" s="35"/>
       <c r="B6" s="11" t="s">
         <v>9</v>
       </c>
@@ -2050,7 +2050,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="36"/>
+      <c r="A7" s="35"/>
       <c r="B7" s="16" t="s">
         <v>9</v>
       </c>
@@ -2077,7 +2077,7 @@
       </c>
     </row>
     <row r="8" spans="1:9" s="10" customFormat="1" ht="144" x14ac:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="35" t="s">
         <v>43</v>
       </c>
       <c r="B8" s="5" t="s">
@@ -2106,7 +2106,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="36"/>
+      <c r="A9" s="35"/>
       <c r="B9" s="11" t="s">
         <v>9</v>
       </c>
@@ -2133,7 +2133,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="36"/>
+      <c r="A10" s="35"/>
       <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
@@ -2160,7 +2160,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="36"/>
+      <c r="A11" s="35"/>
       <c r="B11" s="11" t="s">
         <v>44</v>
       </c>
@@ -2187,7 +2187,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="36"/>
+      <c r="A12" s="35"/>
       <c r="B12" s="11" t="s">
         <v>9</v>
       </c>
@@ -2212,7 +2212,7 @@
       <c r="I12" s="15"/>
     </row>
     <row r="13" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="36"/>
+      <c r="A13" s="35"/>
       <c r="B13" s="11" t="s">
         <v>9</v>
       </c>
@@ -2239,7 +2239,7 @@
       </c>
     </row>
     <row r="14" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="36"/>
+      <c r="A14" s="35"/>
       <c r="B14" s="11" t="s">
         <v>9</v>
       </c>
@@ -2266,7 +2266,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="36"/>
+      <c r="A15" s="35"/>
       <c r="B15" s="11" t="s">
         <v>9</v>
       </c>
@@ -2293,7 +2293,7 @@
       </c>
     </row>
     <row r="16" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="36"/>
+      <c r="A16" s="35"/>
       <c r="B16" s="16" t="s">
         <v>9</v>
       </c>
@@ -2320,7 +2320,7 @@
       </c>
     </row>
     <row r="17" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="35" t="s">
         <v>89</v>
       </c>
       <c r="B17" s="5" t="s">
@@ -2349,7 +2349,7 @@
       </c>
     </row>
     <row r="18" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="36"/>
+      <c r="A18" s="35"/>
       <c r="B18" s="11" t="s">
         <v>9</v>
       </c>
@@ -2376,7 +2376,7 @@
       </c>
     </row>
     <row r="19" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="36"/>
+      <c r="A19" s="35"/>
       <c r="B19" s="11" t="s">
         <v>9</v>
       </c>
@@ -2401,7 +2401,7 @@
       <c r="I19" s="15"/>
     </row>
     <row r="20" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="36"/>
+      <c r="A20" s="35"/>
       <c r="B20" s="11" t="s">
         <v>44</v>
       </c>
@@ -2428,7 +2428,7 @@
       </c>
     </row>
     <row r="21" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="36"/>
+      <c r="A21" s="35"/>
       <c r="B21" s="11" t="s">
         <v>44</v>
       </c>
@@ -2455,7 +2455,7 @@
       </c>
     </row>
     <row r="22" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="36"/>
+      <c r="A22" s="35"/>
       <c r="B22" s="16" t="s">
         <v>112</v>
       </c>
@@ -2482,7 +2482,7 @@
       </c>
     </row>
     <row r="23" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="36" t="s">
+      <c r="A23" s="35" t="s">
         <v>118</v>
       </c>
       <c r="B23" s="5" t="s">
@@ -2511,7 +2511,7 @@
       </c>
     </row>
     <row r="24" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="36"/>
+      <c r="A24" s="35"/>
       <c r="B24" s="11" t="s">
         <v>112</v>
       </c>
@@ -2538,7 +2538,7 @@
       </c>
     </row>
     <row r="25" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="36"/>
+      <c r="A25" s="35"/>
       <c r="B25" s="11" t="s">
         <v>112</v>
       </c>
@@ -2565,7 +2565,7 @@
       </c>
     </row>
     <row r="26" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="36"/>
+      <c r="A26" s="35"/>
       <c r="B26" s="11" t="s">
         <v>112</v>
       </c>
@@ -2592,7 +2592,7 @@
       </c>
     </row>
     <row r="27" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="36"/>
+      <c r="A27" s="35"/>
       <c r="B27" s="16" t="s">
         <v>44</v>
       </c>
@@ -2619,7 +2619,7 @@
       </c>
     </row>
     <row r="28" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="35" t="s">
         <v>145</v>
       </c>
       <c r="B28" s="5" t="s">
@@ -2648,7 +2648,7 @@
       </c>
     </row>
     <row r="29" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="36"/>
+      <c r="A29" s="35"/>
       <c r="B29" s="16" t="s">
         <v>112</v>
       </c>
@@ -2675,7 +2675,7 @@
       </c>
     </row>
     <row r="30" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="36" t="s">
+      <c r="A30" s="35" t="s">
         <v>157</v>
       </c>
       <c r="B30" s="5" t="s">
@@ -2704,7 +2704,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="36"/>
+      <c r="A31" s="35"/>
       <c r="B31" s="11" t="s">
         <v>112</v>
       </c>
@@ -2729,7 +2729,7 @@
       <c r="I31" s="15"/>
     </row>
     <row r="32" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="36"/>
+      <c r="A32" s="35"/>
       <c r="B32" s="11" t="s">
         <v>112</v>
       </c>
@@ -2756,7 +2756,7 @@
       </c>
     </row>
     <row r="33" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="36"/>
+      <c r="A33" s="35"/>
       <c r="B33" s="11" t="s">
         <v>112</v>
       </c>
@@ -2783,7 +2783,7 @@
       </c>
     </row>
     <row r="34" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="36"/>
+      <c r="A34" s="35"/>
       <c r="B34" s="11" t="s">
         <v>9</v>
       </c>
@@ -2810,7 +2810,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="36"/>
+      <c r="A35" s="35"/>
       <c r="B35" s="11" t="s">
         <v>112</v>
       </c>
@@ -2837,7 +2837,7 @@
       </c>
     </row>
     <row r="36" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="36"/>
+      <c r="A36" s="35"/>
       <c r="B36" s="16" t="s">
         <v>112</v>
       </c>
@@ -2864,7 +2864,7 @@
       </c>
     </row>
     <row r="37" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="37" t="s">
+      <c r="A37" s="38" t="s">
         <v>190</v>
       </c>
       <c r="B37" s="5" t="s">
@@ -2893,7 +2893,7 @@
       </c>
     </row>
     <row r="38" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="37"/>
+      <c r="A38" s="38"/>
       <c r="B38" s="11" t="s">
         <v>44</v>
       </c>
@@ -2920,7 +2920,7 @@
       </c>
     </row>
     <row r="39" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="37"/>
+      <c r="A39" s="38"/>
       <c r="B39" s="11" t="s">
         <v>44</v>
       </c>
@@ -2947,7 +2947,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="37"/>
+      <c r="A40" s="38"/>
       <c r="B40" s="11" t="s">
         <v>44</v>
       </c>
@@ -2974,7 +2974,7 @@
       </c>
     </row>
     <row r="41" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="37"/>
+      <c r="A41" s="38"/>
       <c r="B41" s="11" t="s">
         <v>44</v>
       </c>
@@ -3001,7 +3001,7 @@
       </c>
     </row>
     <row r="42" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="37"/>
+      <c r="A42" s="38"/>
       <c r="B42" s="16" t="s">
         <v>112</v>
       </c>
@@ -3028,7 +3028,7 @@
       </c>
     </row>
     <row r="43" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="36" t="s">
+      <c r="A43" s="35" t="s">
         <v>218</v>
       </c>
       <c r="B43" s="5" t="s">
@@ -3057,7 +3057,7 @@
       </c>
     </row>
     <row r="44" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="36"/>
+      <c r="A44" s="35"/>
       <c r="B44" s="11" t="s">
         <v>9</v>
       </c>
@@ -3084,7 +3084,7 @@
       </c>
     </row>
     <row r="45" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="36"/>
+      <c r="A45" s="35"/>
       <c r="B45" s="16" t="s">
         <v>9</v>
       </c>
@@ -3111,7 +3111,7 @@
       </c>
     </row>
     <row r="46" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="35" t="s">
         <v>236</v>
       </c>
       <c r="B46" s="5" t="s">
@@ -3140,7 +3140,7 @@
       </c>
     </row>
     <row r="47" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="36"/>
+      <c r="A47" s="35"/>
       <c r="B47" s="11" t="s">
         <v>44</v>
       </c>
@@ -3167,7 +3167,7 @@
       </c>
     </row>
     <row r="48" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="36"/>
+      <c r="A48" s="35"/>
       <c r="B48" s="11" t="s">
         <v>9</v>
       </c>
@@ -3194,7 +3194,7 @@
       </c>
     </row>
     <row r="49" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="36"/>
+      <c r="A49" s="35"/>
       <c r="B49" s="11" t="s">
         <v>9</v>
       </c>
@@ -3221,7 +3221,7 @@
       </c>
     </row>
     <row r="50" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="36"/>
+      <c r="A50" s="35"/>
       <c r="B50" s="11" t="s">
         <v>9</v>
       </c>
@@ -3248,7 +3248,7 @@
       </c>
     </row>
     <row r="51" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="36"/>
+      <c r="A51" s="35"/>
       <c r="B51" s="11" t="s">
         <v>9</v>
       </c>
@@ -3275,7 +3275,7 @@
       </c>
     </row>
     <row r="52" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="36"/>
+      <c r="A52" s="35"/>
       <c r="B52" s="11" t="s">
         <v>9</v>
       </c>
@@ -3302,7 +3302,7 @@
       </c>
     </row>
     <row r="53" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="36"/>
+      <c r="A53" s="35"/>
       <c r="B53" s="11" t="s">
         <v>9</v>
       </c>
@@ -3329,7 +3329,7 @@
       </c>
     </row>
     <row r="54" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="36"/>
+      <c r="A54" s="35"/>
       <c r="B54" s="11" t="s">
         <v>9</v>
       </c>
@@ -3356,7 +3356,7 @@
       </c>
     </row>
     <row r="55" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="36"/>
+      <c r="A55" s="35"/>
       <c r="B55" s="11" t="s">
         <v>9</v>
       </c>
@@ -3383,7 +3383,7 @@
       </c>
     </row>
     <row r="56" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="36"/>
+      <c r="A56" s="35"/>
       <c r="B56" s="11" t="s">
         <v>9</v>
       </c>
@@ -3410,7 +3410,7 @@
       </c>
     </row>
     <row r="57" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="36" t="s">
+      <c r="A57" s="35" t="s">
         <v>294</v>
       </c>
       <c r="B57" s="5" t="s">
@@ -3439,7 +3439,7 @@
       </c>
     </row>
     <row r="58" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="36"/>
+      <c r="A58" s="35"/>
       <c r="B58" s="11" t="s">
         <v>9</v>
       </c>
@@ -3466,7 +3466,7 @@
       </c>
     </row>
     <row r="59" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="36"/>
+      <c r="A59" s="35"/>
       <c r="B59" s="11" t="s">
         <v>9</v>
       </c>
@@ -3493,7 +3493,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="36"/>
+      <c r="A60" s="35"/>
       <c r="B60" s="16" t="s">
         <v>44</v>
       </c>
@@ -3520,7 +3520,7 @@
       </c>
     </row>
     <row r="61" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="36" t="s">
+      <c r="A61" s="35" t="s">
         <v>318</v>
       </c>
       <c r="B61" s="21" t="s">
@@ -3549,7 +3549,7 @@
       </c>
     </row>
     <row r="62" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="36"/>
+      <c r="A62" s="35"/>
       <c r="B62" s="11" t="s">
         <v>9</v>
       </c>
@@ -3576,7 +3576,7 @@
       </c>
     </row>
     <row r="63" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="36"/>
+      <c r="A63" s="35"/>
       <c r="B63" s="11" t="s">
         <v>9</v>
       </c>
@@ -3603,7 +3603,7 @@
       </c>
     </row>
     <row r="64" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="36"/>
+      <c r="A64" s="35"/>
       <c r="B64" s="11" t="s">
         <v>9</v>
       </c>
@@ -3630,7 +3630,7 @@
       </c>
     </row>
     <row r="65" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="36"/>
+      <c r="A65" s="35"/>
       <c r="B65" s="11" t="s">
         <v>9</v>
       </c>
@@ -3657,7 +3657,7 @@
       </c>
     </row>
     <row r="66" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="36"/>
+      <c r="A66" s="35"/>
       <c r="B66" s="11" t="s">
         <v>9</v>
       </c>
@@ -3684,7 +3684,7 @@
       </c>
     </row>
     <row r="67" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="36"/>
+      <c r="A67" s="35"/>
       <c r="B67" s="11" t="s">
         <v>44</v>
       </c>
@@ -3711,7 +3711,7 @@
       </c>
     </row>
     <row r="68" spans="1:9" s="10" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="36"/>
+      <c r="A68" s="35"/>
       <c r="B68" s="26" t="s">
         <v>44</v>
       </c>
@@ -3744,14 +3744,14 @@
       <c r="G69" s="28"/>
     </row>
     <row r="70" spans="1:9" s="4" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="35" t="s">
+      <c r="A70" s="37" t="s">
         <v>359</v>
       </c>
-      <c r="B70" s="35"/>
-      <c r="C70" s="35"/>
-      <c r="D70" s="35"/>
-      <c r="E70" s="35"/>
-      <c r="F70" s="35"/>
+      <c r="B70" s="37"/>
+      <c r="C70" s="37"/>
+      <c r="D70" s="37"/>
+      <c r="E70" s="37"/>
+      <c r="F70" s="37"/>
       <c r="G70" s="28"/>
     </row>
     <row r="71" spans="1:9" s="4" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.15">
@@ -3820,12 +3820,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="A8:A16"/>
-    <mergeCell ref="A17:A22"/>
-    <mergeCell ref="A23:A27"/>
     <mergeCell ref="A70:F70"/>
     <mergeCell ref="A30:A36"/>
     <mergeCell ref="A37:A42"/>
@@ -3833,6 +3827,12 @@
     <mergeCell ref="A46:A56"/>
     <mergeCell ref="A57:A60"/>
     <mergeCell ref="A61:A68"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="A8:A16"/>
+    <mergeCell ref="A17:A22"/>
+    <mergeCell ref="A23:A27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>